<commit_message>
Update ReadMe inside of the Excel file
</commit_message>
<xml_diff>
--- a/Combined Tax Estimator.xlsx
+++ b/Combined Tax Estimator.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ab913e7457364688/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{13B519AE-AB73-40E7-9524-407E8959D0D7}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{F3B28514-71F1-41DD-9E29-9270D63E5505}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="18636" yWindow="492" windowWidth="26892" windowHeight="22536" xr2:uid="{F29755CA-56C7-4287-B0E1-95271A5704F5}"/>
   </bookViews>
@@ -69,12 +69,18 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="358" uniqueCount="154">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="360" uniqueCount="156">
   <si>
     <t xml:space="preserve">Purpose </t>
   </si>
   <si>
     <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
       <t xml:space="preserve">This spreadsheet helps you quickly estimate your total federal tax liability by combining the most common tax types for employed individuals in one place.
 </t>
     </r>
@@ -82,9 +88,8 @@
       <rPr>
         <u/>
         <sz val="11"/>
-        <color theme="1"/>
+        <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>Key benefit of this calculator</t>
@@ -92,9 +97,8 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color theme="1"/>
+        <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">:
@@ -105,23 +109,21 @@
       <rPr>
         <b/>
         <sz val="11"/>
-        <color theme="1"/>
+        <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t>This tool calculates and properly combines most common tax types:</t>
+      <t xml:space="preserve">This tool calculates and properly combines most common tax types:
+</t>
     </r>
     <r>
       <rPr>
         <sz val="11"/>
-        <color theme="1"/>
+        <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">
-  - Federal Income Tax (including Alternative Minimum Tax (AMT))
+      <t xml:space="preserve">  - Federal Income Tax (including Alternative Minimum Tax (AMT))
   - Long-Term Capital Gains Tax
   - Social Security Tax
   - Medicare Taxes (including Additional Medicare Tax and NIIT)
@@ -131,9 +133,8 @@
       <rPr>
         <b/>
         <sz val="11"/>
-        <color theme="1"/>
+        <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>Philosophy:</t>
@@ -141,9 +142,8 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color theme="1"/>
+        <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> This is an estimation tool, not a precise calculator. It intentionally omits some deductions to keep things simple. It's better to slightly overestimate (and get a refund) than underestimate (and face penalties).</t>
@@ -157,20 +157,118 @@
       <rPr>
         <b/>
         <sz val="11"/>
-        <color theme="1"/>
+        <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">Input Your Income ('Estomator' tab, </t>
+      <t xml:space="preserve">1. If you are viewing the public read-only version, get your own private copy of the calculator:
+</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">  - Go to: </t>
     </r>
     <r>
       <rPr>
         <b/>
         <sz val="11"/>
-        <color theme="5"/>
+        <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
-        <family val="2"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>File</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve"> &gt; </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Create a Copy</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>.
+    To use with Excel for Desktop (Windows or Mac), select '</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Download a Copy</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>'.
+    To use with Excel Online (free), select '</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t>Create a copy online'</t>
+    </r>
+    <r>
+      <rPr>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">.
+  - Alternatively, download the calculator Excel file directly from the GitHub repo (link below).
+</t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FF000000"/>
+        <rFont val="Aptos Narrow"/>
+        <scheme val="minor"/>
+      </rPr>
+      <t xml:space="preserve">2. Input Your Income ('Estomator' tab, </t>
+    </r>
+    <r>
+      <rPr>
+        <b/>
+        <sz val="11"/>
+        <color rgb="FFE97132"/>
+        <rFont val="Aptos Narrow"/>
         <scheme val="minor"/>
       </rPr>
       <t>orange</t>
@@ -179,23 +277,21 @@
       <rPr>
         <b/>
         <sz val="11"/>
-        <color theme="1"/>
+        <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve"> cells only):</t>
+      <t xml:space="preserve"> cells only):
+</t>
     </r>
     <r>
       <rPr>
         <sz val="11"/>
-        <color theme="1"/>
+        <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">
-  - Enter your estimated income in section 'Your extimated income'.
+      <t xml:space="preserve">  - Enter your estimated income in section 'Your extimated income'.
   - Each income category has 3 input fields. Use them however you like (they're simply added together).
   - Only edit </t>
     </r>
@@ -203,9 +299,8 @@
       <rPr>
         <b/>
         <sz val="11"/>
-        <color theme="5"/>
+        <color rgb="FFE97132"/>
         <rFont val="Aptos Narrow"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>orange</t>
@@ -213,9 +308,8 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color theme="1"/>
+        <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> cells. All other cells are auto-computed.
@@ -226,20 +320,18 @@
       <rPr>
         <b/>
         <sz val="11"/>
-        <color theme="1"/>
+        <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
-      <t xml:space="preserve">Review Your Results:
+      <t xml:space="preserve">3. Review Your Results:
 </t>
     </r>
     <r>
       <rPr>
         <sz val="11"/>
-        <color theme="1"/>
+        <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve">  - </t>
@@ -248,9 +340,8 @@
       <rPr>
         <b/>
         <sz val="11"/>
-        <color theme="1"/>
+        <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>'Total Tax Summary' section:</t>
@@ -258,9 +349,8 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color theme="1"/>
+        <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> View estimated tax by type and your total.
@@ -270,9 +360,8 @@
       <rPr>
         <b/>
         <sz val="11"/>
-        <color theme="1"/>
+        <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>Detail sections below:</t>
@@ -280,9 +369,8 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color theme="1"/>
+        <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> See exactly how each tax is calculated.
@@ -292,9 +380,8 @@
       <rPr>
         <b/>
         <sz val="11"/>
-        <color theme="1"/>
+        <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t>'Parameters' tab:</t>
@@ -302,13 +389,18 @@
     <r>
       <rPr>
         <sz val="11"/>
-        <color theme="1"/>
+        <color rgb="FF000000"/>
         <rFont val="Aptos Narrow"/>
-        <family val="2"/>
         <scheme val="minor"/>
       </rPr>
       <t xml:space="preserve"> Reference tax rates and brackets for each year.</t>
     </r>
+  </si>
+  <si>
+    <t>Link to this calculator on GitHub:</t>
+  </si>
+  <si>
+    <t>https://github.com/macrogreg/Combined-Income-Tax-Estimator</t>
   </si>
   <si>
     <t>Tax types not considered</t>
@@ -886,7 +978,7 @@
     <numFmt numFmtId="167" formatCode="0.0%"/>
     <numFmt numFmtId="168" formatCode="_(&quot;$&quot;* #,##0_);_(&quot;$&quot;* \(#,##0\);_(&quot;$&quot;* &quot;-&quot;??_);_(@_)"/>
   </numFmts>
-  <fonts count="31">
+  <fonts count="36">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -1106,19 +1198,51 @@
       <scheme val="minor"/>
     </font>
     <font>
-      <b/>
+      <u/>
       <sz val="11"/>
-      <color theme="5"/>
+      <color theme="10"/>
       <name val="Aptos Narrow"/>
       <family val="2"/>
       <scheme val="minor"/>
     </font>
     <font>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <u/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FF000000"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color rgb="FFE97132"/>
+      <name val="Aptos Narrow"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
       <sz val="11"/>
       <color theme="1"/>
       <name val="Aptos Narrow"/>
-      <family val="2"/>
+      <scheme val="minor"/>
+    </font>
+    <font>
+      <b/>
+      <sz val="11"/>
+      <color theme="1"/>
+      <name val="Aptos Narrow"/>
       <scheme val="minor"/>
     </font>
   </fonts>
@@ -1308,7 +1432,7 @@
       <diagonal/>
     </border>
   </borders>
-  <cellStyleXfs count="10">
+  <cellStyleXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
     <xf numFmtId="44" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
@@ -1321,8 +1445,9 @@
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="81">
+  <cellXfs count="85">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1457,14 +1582,27 @@
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyAlignment="1">
       <alignment horizontal="right"/>
     </xf>
+    <xf numFmtId="0" fontId="30" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="34" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="35" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="0" borderId="0" xfId="10" applyFont="1" applyAlignment="1">
+      <alignment vertical="top" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="27" fillId="0" borderId="14" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
   </cellXfs>
-  <cellStyles count="10">
+  <cellStyles count="11">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
     <cellStyle name="Heading 2" xfId="3" builtinId="17"/>
     <cellStyle name="Heading 3" xfId="5" builtinId="18"/>
+    <cellStyle name="Hyperlink" xfId="10" builtinId="8"/>
     <cellStyle name="Input" xfId="4" builtinId="20"/>
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
     <cellStyle name="Percent" xfId="2" builtinId="5"/>
@@ -5305,10 +5443,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C9605775-5D08-4EA7-A2E6-803BF37BCEA6}">
-  <dimension ref="B3:B14"/>
+  <dimension ref="B3:B17"/>
   <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="2" max="2" width="81.140625" style="77" customWidth="1"/>
+    <col min="2" max="2" width="85" style="77" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="2:2" ht="18" thickBot="1">
@@ -5317,7 +5455,7 @@
       </c>
     </row>
     <row r="4" spans="2:2" ht="217.5" customHeight="1" thickTop="1">
-      <c r="B4" s="76" t="s">
+      <c r="B4" s="80" t="s">
         <v>1</v>
       </c>
     </row>
@@ -5326,32 +5464,46 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="2:2" ht="188.25" customHeight="1" thickTop="1">
-      <c r="B7" s="76" t="s">
+    <row r="7" spans="2:2" ht="298.5" customHeight="1" thickTop="1">
+      <c r="B7" s="81" t="s">
         <v>3</v>
       </c>
     </row>
-    <row r="9" spans="2:2" ht="15" thickBot="1">
-      <c r="B9" s="78" t="s">
+    <row r="8" spans="2:2" ht="15">
+      <c r="B8" s="82" t="s">
         <v>4</v>
       </c>
     </row>
-    <row r="10" spans="2:2" ht="101.25" customHeight="1">
-      <c r="B10" s="76" t="s">
+    <row r="9" spans="2:2" ht="15">
+      <c r="B9" s="83" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="13" spans="2:2" ht="15" thickBot="1">
-      <c r="B13" s="78" t="s">
+    <row r="11" spans="2:2" ht="15" thickBot="1">
+      <c r="B11" s="78" t="s">
         <v>6</v>
       </c>
     </row>
-    <row r="14" spans="2:2" ht="81.75" customHeight="1">
-      <c r="B14" s="76" t="s">
+    <row r="12" spans="2:2" ht="101.25" customHeight="1">
+      <c r="B12" s="76" t="s">
         <v>7</v>
       </c>
     </row>
+    <row r="15" spans="2:2" ht="15" thickBot="1">
+      <c r="B15" s="78" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="16" spans="2:2" ht="81.75" customHeight="1">
+      <c r="B16" s="76" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17" ht="15"/>
   </sheetData>
+  <hyperlinks>
+    <hyperlink ref="B9" r:id="rId1" xr:uid="{AF5B704B-2169-4D38-B0A1-DEA648950453}"/>
+  </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
 </file>
@@ -5374,27 +5526,27 @@
   <sheetData>
     <row r="2" spans="2:12" s="30" customFormat="1" ht="15.6">
       <c r="B2" s="23" t="s">
-        <v>8</v>
+        <v>10</v>
       </c>
       <c r="C2"/>
       <c r="F2" s="65" t="s">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="G2"/>
     </row>
     <row r="3" spans="2:12" s="30" customFormat="1" ht="15.6">
       <c r="B3" s="23" t="s">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="C3"/>
       <c r="F3" s="64" t="s">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="G3"/>
     </row>
     <row r="5" spans="2:12" ht="18" thickBot="1">
       <c r="B5" s="15" t="s">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="C5" s="15"/>
       <c r="D5" s="15"/>
@@ -5407,26 +5559,26 @@
       <c r="K5" s="15"/>
     </row>
     <row r="6" spans="2:12" ht="15" thickTop="1">
-      <c r="B6" s="80" t="s">
-        <v>13</v>
-      </c>
-      <c r="C6" s="80"/>
+      <c r="B6" s="84" t="s">
+        <v>15</v>
+      </c>
+      <c r="C6" s="84"/>
     </row>
     <row r="7" spans="2:12">
       <c r="B7" s="67"/>
     </row>
     <row r="8" spans="2:12">
       <c r="B8" s="3" t="s">
-        <v>14</v>
+        <v>16</v>
       </c>
       <c r="C8" s="8">
         <v>2025</v>
       </c>
       <c r="F8" s="3" t="s">
-        <v>15</v>
+        <v>17</v>
       </c>
       <c r="G8" s="8" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
     </row>
     <row r="9" spans="2:12">
@@ -5436,64 +5588,64 @@
     </row>
     <row r="10" spans="2:12" ht="15" thickBot="1">
       <c r="B10" s="37" t="s">
-        <v>17</v>
+        <v>19</v>
       </c>
       <c r="C10" s="37"/>
       <c r="D10" s="12"/>
       <c r="F10" s="37" t="s">
-        <v>18</v>
+        <v>20</v>
       </c>
       <c r="G10" s="37"/>
       <c r="J10" s="37" t="s">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="K10" s="37"/>
     </row>
     <row r="11" spans="2:12">
       <c r="B11" s="26" t="s">
-        <v>20</v>
+        <v>22</v>
       </c>
       <c r="D11" s="12"/>
       <c r="F11" s="26" t="s">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="J11" s="26" t="s">
-        <v>22</v>
+        <v>24</v>
       </c>
     </row>
     <row r="13" spans="2:12">
       <c r="B13" t="s">
-        <v>23</v>
+        <v>25</v>
       </c>
       <c r="C13" s="9">
         <v>80000</v>
       </c>
       <c r="F13" t="s">
-        <v>24</v>
+        <v>26</v>
       </c>
       <c r="G13" s="9">
         <v>5000</v>
       </c>
       <c r="J13" s="46" t="s">
-        <v>25</v>
+        <v>27</v>
       </c>
       <c r="K13" s="42"/>
     </row>
     <row r="14" spans="2:12">
       <c r="B14" t="s">
-        <v>26</v>
+        <v>28</v>
       </c>
       <c r="C14" s="9">
         <v>0</v>
       </c>
       <c r="F14" t="s">
-        <v>27</v>
+        <v>29</v>
       </c>
       <c r="G14" s="9">
         <v>0</v>
       </c>
       <c r="J14" t="s">
-        <v>28</v>
+        <v>30</v>
       </c>
       <c r="K14" s="2">
         <f>_xlfn.XLOOKUP(TRUE, StandardDeductionAmountTable[IsSelected], StandardDeductionAmountTable[Standard 
@@ -5503,30 +5655,30 @@
     </row>
     <row r="15" spans="2:12" ht="15" thickBot="1">
       <c r="B15" s="10" t="s">
-        <v>29</v>
+        <v>31</v>
       </c>
       <c r="C15" s="11">
         <v>0</v>
       </c>
       <c r="F15" s="10" t="s">
-        <v>30</v>
+        <v>32</v>
       </c>
       <c r="G15" s="11">
         <v>0</v>
       </c>
       <c r="J15" s="10" t="s">
-        <v>31</v>
+        <v>33</v>
       </c>
       <c r="K15" s="11">
         <v>0</v>
       </c>
       <c r="L15" s="43" t="s">
-        <v>32</v>
+        <v>34</v>
       </c>
     </row>
     <row r="16" spans="2:12">
       <c r="B16" s="3" t="s">
-        <v>33</v>
+        <v>35</v>
       </c>
       <c r="C16" s="4">
         <f>SUM(C13:C15)</f>
@@ -5541,7 +5693,7 @@
         <v>✔</v>
       </c>
       <c r="F16" s="3" t="s">
-        <v>34</v>
+        <v>36</v>
       </c>
       <c r="G16" s="4">
         <f>SUM(G13:G15)</f>
@@ -5556,7 +5708,7 @@
         <v>✔</v>
       </c>
       <c r="J16" s="3" t="s">
-        <v>35</v>
+        <v>37</v>
       </c>
       <c r="K16" s="4">
         <f xml:space="preserve"> MAX(K14:K15)</f>
@@ -5573,27 +5725,27 @@
     </row>
     <row r="19" spans="2:12" ht="15" thickBot="1">
       <c r="B19" s="37" t="s">
-        <v>36</v>
+        <v>38</v>
       </c>
       <c r="C19" s="37"/>
       <c r="F19" s="37" t="s">
-        <v>37</v>
+        <v>39</v>
       </c>
       <c r="G19" s="37"/>
       <c r="J19" s="37" t="s">
-        <v>38</v>
+        <v>40</v>
       </c>
       <c r="K19" s="37"/>
     </row>
     <row r="20" spans="2:12">
       <c r="B20" s="26" t="s">
-        <v>39</v>
+        <v>41</v>
       </c>
       <c r="F20" s="26" t="s">
-        <v>40</v>
+        <v>42</v>
       </c>
       <c r="J20" s="26" t="s">
-        <v>41</v>
+        <v>43</v>
       </c>
     </row>
     <row r="21" spans="2:12">
@@ -5602,19 +5754,19 @@
     </row>
     <row r="22" spans="2:12">
       <c r="B22" t="s">
-        <v>42</v>
+        <v>44</v>
       </c>
       <c r="C22" s="9">
         <v>10000</v>
       </c>
       <c r="F22" t="s">
-        <v>43</v>
+        <v>45</v>
       </c>
       <c r="G22" s="9">
         <v>5000</v>
       </c>
       <c r="J22" t="s">
-        <v>44</v>
+        <v>46</v>
       </c>
       <c r="K22" s="9">
         <v>2000</v>
@@ -5622,19 +5774,19 @@
     </row>
     <row r="23" spans="2:12">
       <c r="B23" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
       <c r="C23" s="9">
         <v>0</v>
       </c>
       <c r="F23" t="s">
-        <v>46</v>
+        <v>48</v>
       </c>
       <c r="G23" s="9">
         <v>0</v>
       </c>
       <c r="J23" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
       <c r="K23" s="9">
         <v>0</v>
@@ -5642,19 +5794,19 @@
     </row>
     <row r="24" spans="2:12" ht="15" thickBot="1">
       <c r="B24" s="10" t="s">
-        <v>48</v>
+        <v>50</v>
       </c>
       <c r="C24" s="11">
         <v>0</v>
       </c>
       <c r="F24" s="10" t="s">
-        <v>49</v>
+        <v>51</v>
       </c>
       <c r="G24" s="11">
         <v>0</v>
       </c>
       <c r="J24" s="10" t="s">
-        <v>50</v>
+        <v>52</v>
       </c>
       <c r="K24" s="11">
         <v>0</v>
@@ -5662,7 +5814,7 @@
     </row>
     <row r="25" spans="2:12">
       <c r="B25" s="3" t="s">
-        <v>51</v>
+        <v>53</v>
       </c>
       <c r="C25" s="4">
         <f>SUM(C22:C24)</f>
@@ -5677,7 +5829,7 @@
         <v>✔</v>
       </c>
       <c r="F25" s="3" t="s">
-        <v>52</v>
+        <v>54</v>
       </c>
       <c r="G25" s="4">
         <f>SUM(G22:G24)</f>
@@ -5692,7 +5844,7 @@
         <v>✔</v>
       </c>
       <c r="J25" s="3" t="s">
-        <v>53</v>
+        <v>55</v>
       </c>
       <c r="K25" s="4">
         <f>SUM(K22:K24)</f>
@@ -5725,7 +5877,7 @@
     </row>
     <row r="28" spans="2:12" ht="18" thickBot="1">
       <c r="B28" s="39" t="s">
-        <v>54</v>
+        <v>56</v>
       </c>
       <c r="C28" s="39"/>
       <c r="D28" s="40"/>
@@ -5738,10 +5890,10 @@
       <c r="K28" s="39"/>
     </row>
     <row r="29" spans="2:12" ht="15" thickTop="1">
-      <c r="B29" s="80" t="s">
-        <v>55</v>
-      </c>
-      <c r="C29" s="80"/>
+      <c r="B29" s="84" t="s">
+        <v>57</v>
+      </c>
+      <c r="C29" s="84"/>
     </row>
     <row r="30" spans="2:12">
       <c r="B30" s="38"/>
@@ -5749,11 +5901,11 @@
     </row>
     <row r="31" spans="2:12" ht="15" thickBot="1">
       <c r="B31" s="37" t="s">
-        <v>56</v>
+        <v>58</v>
       </c>
       <c r="C31" s="37"/>
       <c r="F31" s="37" t="s">
-        <v>57</v>
+        <v>59</v>
       </c>
       <c r="G31" s="41"/>
     </row>
@@ -5887,7 +6039,7 @@
     </row>
     <row r="37" spans="2:11" ht="15" thickBot="1">
       <c r="B37" s="3" t="s">
-        <v>58</v>
+        <v>60</v>
       </c>
       <c r="C37" s="4">
         <f xml:space="preserve"> SUM(C33:C36)</f>
@@ -5922,7 +6074,7 @@
     </row>
     <row r="38" spans="2:11">
       <c r="F38" s="3" t="s">
-        <v>59</v>
+        <v>61</v>
       </c>
       <c r="G38" s="4">
         <f>SUM(G33:G37)</f>
@@ -5943,7 +6095,7 @@
     </row>
     <row r="40" spans="2:11" ht="18" thickBot="1">
       <c r="B40" s="39" t="s">
-        <v>60</v>
+        <v>62</v>
       </c>
       <c r="C40" s="39"/>
       <c r="D40" s="40"/>
@@ -5956,18 +6108,18 @@
       <c r="K40" s="39"/>
     </row>
     <row r="41" spans="2:11" ht="15" thickTop="1">
-      <c r="B41" s="80" t="s">
-        <v>61</v>
-      </c>
-      <c r="C41" s="80"/>
+      <c r="B41" s="84" t="s">
+        <v>63</v>
+      </c>
+      <c r="C41" s="84"/>
     </row>
     <row r="43" spans="2:11" ht="15" thickBot="1">
       <c r="B43" s="37" t="s">
-        <v>62</v>
+        <v>64</v>
       </c>
       <c r="C43" s="37"/>
       <c r="F43" s="37" t="s">
-        <v>63</v>
+        <v>65</v>
       </c>
       <c r="G43" s="37"/>
     </row>
@@ -5977,10 +6129,10 @@
     </row>
     <row r="45" spans="2:11">
       <c r="B45" t="s">
-        <v>64</v>
+        <v>66</v>
       </c>
       <c r="C45" s="2" t="s">
-        <v>65</v>
+        <v>67</v>
       </c>
       <c r="F45" s="48" t="str">
         <f xml:space="preserve"> $B$37</f>
@@ -6052,7 +6204,7 @@
         <v>= $C$121</v>
       </c>
       <c r="F47" s="70" t="s">
-        <v>66</v>
+        <v>68</v>
       </c>
       <c r="G47" s="73">
         <f xml:space="preserve"> G46 / G45</f>
@@ -6087,7 +6239,7 @@
         <v>= $K$64</v>
       </c>
       <c r="F48" s="50" t="s">
-        <v>67</v>
+        <v>69</v>
       </c>
       <c r="G48" s="74">
         <f xml:space="preserve"> G45 - G46</f>
@@ -6151,7 +6303,7 @@
     </row>
     <row r="51" spans="2:12" ht="15.6">
       <c r="B51" s="31" t="s">
-        <v>68</v>
+        <v>70</v>
       </c>
       <c r="C51" s="32">
         <f xml:space="preserve"> SUBTOTAL(109,TotalTaxEstimateTable[Amount])</f>
@@ -6160,7 +6312,7 @@
     </row>
     <row r="55" spans="2:12" ht="18" thickBot="1">
       <c r="B55" s="15" t="s">
-        <v>69</v>
+        <v>71</v>
       </c>
       <c r="C55" s="15"/>
       <c r="D55" s="15"/>
@@ -6175,21 +6327,21 @@
     <row r="56" spans="2:12" ht="15" thickTop="1"/>
     <row r="57" spans="2:12" ht="15" thickBot="1">
       <c r="B57" s="37" t="s">
-        <v>70</v>
+        <v>72</v>
       </c>
       <c r="C57" s="37"/>
       <c r="F57" s="37" t="s">
-        <v>71</v>
+        <v>73</v>
       </c>
       <c r="G57" s="37"/>
       <c r="J57" s="37" t="s">
-        <v>72</v>
+        <v>74</v>
       </c>
       <c r="K57" s="37"/>
     </row>
     <row r="59" spans="2:12">
       <c r="B59" s="52" t="s">
-        <v>73</v>
+        <v>75</v>
       </c>
       <c r="C59" s="53">
         <f xml:space="preserve"> $C$16</f>
@@ -6206,7 +6358,7 @@
         <v>= $C$16</v>
       </c>
       <c r="F59" t="s">
-        <v>74</v>
+        <v>76</v>
       </c>
       <c r="G59" s="2">
         <f>$C$25 + $G$25 + $K$25</f>
@@ -6221,7 +6373,7 @@
         <v>✔</v>
       </c>
       <c r="J59" t="s">
-        <v>75</v>
+        <v>77</v>
       </c>
       <c r="K59" s="2">
         <f>_xlfn.XLOOKUP(TRUE, SocialSecurityTaxRateTable[IsSelected], SocialSecurityTaxRateTable[Max Taxable Income], NotFoundLabelCell)</f>
@@ -6249,7 +6401,7 @@
     <row r="60" spans="2:12">
       <c r="C60" s="2"/>
       <c r="F60" t="s">
-        <v>76</v>
+        <v>78</v>
       </c>
       <c r="G60" s="2">
         <f xml:space="preserve"> $C$37</f>
@@ -6268,7 +6420,7 @@
     </row>
     <row r="61" spans="2:12">
       <c r="B61" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C61" s="6">
         <f>_xlfn.XLOOKUP(TRUE, MedicareWageTaxRateTable[IsSelected], MedicareWageTaxRateTable[Medicare Rate], NotFoundLabelCell)</f>
@@ -6293,7 +6445,7 @@
         <v>in MedicareWageTaxRateTable</v>
       </c>
       <c r="J61" t="s">
-        <v>78</v>
+        <v>80</v>
       </c>
       <c r="K61" s="6">
         <f>_xlfn.XLOOKUP(TRUE, SocialSecurityTaxRateTable[IsSelected], SocialSecurityTaxRateTable[SocialSecurity Rate], NotFoundLabelCell)</f>
@@ -6320,7 +6472,7 @@
     </row>
     <row r="62" spans="2:12">
       <c r="B62" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C62" s="2">
         <f>_xlfn.XLOOKUP(TRUE, MedicareWageTaxRateTable[IsSelected], MedicareWageTaxRateTable[RangeStart], NotFoundLabelCell)</f>
@@ -6345,7 +6497,7 @@
         <v>in MedicareWageTaxRateTable</v>
       </c>
       <c r="F62" t="s">
-        <v>80</v>
+        <v>82</v>
       </c>
       <c r="G62" s="2">
         <f>_xlfn.XLOOKUP(TRUE, MedicareNetInvestIncomeTaxTable[IsSelected], MedicareNetInvestIncomeTaxTable[Modified AGI Threshold], NotFoundLabelCell)</f>
@@ -6370,7 +6522,7 @@
         <v>in MedicareNetInvestIncomeTaxTable</v>
       </c>
       <c r="J62" t="s">
-        <v>81</v>
+        <v>83</v>
       </c>
       <c r="K62" s="2">
         <f xml:space="preserve"> MIN( $C$16, K59 )</f>
@@ -6386,7 +6538,7 @@
     </row>
     <row r="63" spans="2:12">
       <c r="F63" t="s">
-        <v>82</v>
+        <v>84</v>
       </c>
       <c r="G63" s="21" t="b">
         <f xml:space="preserve"> G60 &gt;= G62</f>
@@ -6402,7 +6554,7 @@
     </row>
     <row r="64" spans="2:12">
       <c r="B64" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C64" s="2">
         <f>IF(
@@ -6431,7 +6583,7 @@
         <v>in MedicareWageTaxRateTable</v>
       </c>
       <c r="J64" s="17" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="K64" s="18">
         <f xml:space="preserve"> K62 * K61</f>
@@ -6447,7 +6599,7 @@
     </row>
     <row r="65" spans="2:12">
       <c r="B65" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C65" s="2">
         <f xml:space="preserve"> IF(
@@ -6458,7 +6610,7 @@
         <v>1160</v>
       </c>
       <c r="F65" t="s">
-        <v>86</v>
+        <v>88</v>
       </c>
       <c r="G65" s="6">
         <f>_xlfn.XLOOKUP(TRUE, MedicareNetInvestIncomeTaxTable[IsSelected], MedicareNetInvestIncomeTaxTable[NetInvestInc Rate], NotFoundLabelCell)</f>
@@ -6485,7 +6637,7 @@
     </row>
     <row r="66" spans="2:12">
       <c r="F66" t="s">
-        <v>87</v>
+        <v>89</v>
       </c>
       <c r="G66" s="2">
         <f xml:space="preserve"> IF( G63,
@@ -6497,7 +6649,7 @@
     </row>
     <row r="67" spans="2:12">
       <c r="B67" s="17" t="s">
-        <v>84</v>
+        <v>86</v>
       </c>
       <c r="C67" s="18">
         <f xml:space="preserve"> C64 + C65</f>
@@ -6513,7 +6665,7 @@
     </row>
     <row r="68" spans="2:12">
       <c r="F68" s="17" t="s">
-        <v>88</v>
+        <v>90</v>
       </c>
       <c r="G68" s="18">
         <f xml:space="preserve"> IF(
@@ -6526,7 +6678,7 @@
     </row>
     <row r="71" spans="2:12" ht="18" thickBot="1">
       <c r="B71" s="15" t="s">
-        <v>89</v>
+        <v>91</v>
       </c>
       <c r="C71" s="15"/>
       <c r="D71" s="15"/>
@@ -6541,15 +6693,15 @@
     <row r="72" spans="2:12" ht="15" thickTop="1"/>
     <row r="73" spans="2:12" ht="15" thickBot="1">
       <c r="B73" s="37" t="s">
-        <v>90</v>
+        <v>92</v>
       </c>
       <c r="C73" s="37"/>
       <c r="F73" s="37" t="s">
-        <v>91</v>
+        <v>93</v>
       </c>
       <c r="G73" s="37"/>
       <c r="J73" s="37" t="s">
-        <v>92</v>
+        <v>94</v>
       </c>
       <c r="K73" s="37"/>
     </row>
@@ -6693,14 +6845,14 @@
     </row>
     <row r="78" spans="2:12">
       <c r="B78" s="54" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="C78" s="55">
         <f xml:space="preserve"> SUM(C75:C77)</f>
         <v>92000</v>
       </c>
       <c r="F78" s="54" t="s">
-        <v>93</v>
+        <v>95</v>
       </c>
       <c r="G78" s="55">
         <f>SUM(G75:G77)</f>
@@ -6724,7 +6876,7 @@
     </row>
     <row r="79" spans="2:12">
       <c r="J79" s="51" t="s">
-        <v>94</v>
+        <v>96</v>
       </c>
     </row>
     <row r="80" spans="2:12">
@@ -6785,7 +6937,7 @@
         <v>= - $K$16</v>
       </c>
       <c r="F81" s="54" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="G81" s="55">
         <f xml:space="preserve"> SUM(G80:G80)</f>
@@ -6794,7 +6946,7 @@
     </row>
     <row r="82" spans="2:8">
       <c r="B82" s="54" t="s">
-        <v>95</v>
+        <v>97</v>
       </c>
       <c r="C82" s="55">
         <f xml:space="preserve"> SUM(C80:C81)</f>
@@ -6805,7 +6957,7 @@
       <c r="B83" s="33"/>
       <c r="C83" s="33"/>
       <c r="F83" s="60" t="s">
-        <v>96</v>
+        <v>98</v>
       </c>
       <c r="G83" s="61">
         <f xml:space="preserve"> MAX( G78 + G81, 0 )</f>
@@ -6814,7 +6966,7 @@
     </row>
     <row r="84" spans="2:8">
       <c r="B84" s="52" t="s">
-        <v>97</v>
+        <v>99</v>
       </c>
       <c r="C84" s="53">
         <f xml:space="preserve"> MAX( C78 + C82, 0 )</f>
@@ -6823,7 +6975,7 @@
     </row>
     <row r="85" spans="2:8">
       <c r="F85" t="s">
-        <v>98</v>
+        <v>100</v>
       </c>
       <c r="G85" s="1">
         <f>_xlfn.XLOOKUP(TRUE, AlternativeMimumumTaxThresholdsTable[IsSelected], AlternativeMimumumTaxThresholdsTable[AMT Exemption], NotFoundLabelCell)</f>
@@ -6850,7 +7002,7 @@
     </row>
     <row r="86" spans="2:8">
       <c r="B86" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="C86" s="6">
         <f>_xlfn.XLOOKUP(TRUE, FederalIncomeTaxRateTable[IsSelected], FederalIncomeTaxRateTable[Federal Tax Rate], NotFoundLabelCell)</f>
@@ -6875,7 +7027,7 @@
         <v>in FederalIncomeTaxRateTable</v>
       </c>
       <c r="F86" t="s">
-        <v>99</v>
+        <v>101</v>
       </c>
       <c r="G86" s="1">
         <f>_xlfn.XLOOKUP(TRUE, AlternativeMimumumTaxThresholdsTable[IsSelected], AlternativeMimumumTaxThresholdsTable[Phaseout Threshold], NotFoundLabelCell)</f>
@@ -6902,7 +7054,7 @@
     </row>
     <row r="87" spans="2:8">
       <c r="B87" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="C87" s="2">
         <f>_xlfn.XLOOKUP(TRUE, FederalIncomeTaxRateTable[IsSelected], FederalIncomeTaxRateTable[RangeStart], NotFoundLabelCell)</f>
@@ -6927,7 +7079,7 @@
         <v>in FederalIncomeTaxRateTable</v>
       </c>
       <c r="F87" t="s">
-        <v>100</v>
+        <v>102</v>
       </c>
       <c r="G87" s="2">
         <f xml:space="preserve"> MAX( G83 - G86, 0)</f>
@@ -6936,7 +7088,7 @@
     </row>
     <row r="88" spans="2:8">
       <c r="F88" t="s">
-        <v>101</v>
+        <v>103</v>
       </c>
       <c r="G88" s="2">
         <f>G87 * 0.25</f>
@@ -6945,7 +7097,7 @@
     </row>
     <row r="89" spans="2:8">
       <c r="B89" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="C89" s="2">
         <f>IF(
@@ -6974,7 +7126,7 @@
         <v>in FederalIncomeTaxRateTable</v>
       </c>
       <c r="F89" s="62" t="s">
-        <v>102</v>
+        <v>104</v>
       </c>
       <c r="G89" s="63">
         <f>MAX( G85 - G88, 0 )</f>
@@ -6983,7 +7135,7 @@
     </row>
     <row r="90" spans="2:8">
       <c r="B90" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="C90" s="2">
         <f xml:space="preserve"> IF(
@@ -6998,7 +7150,7 @@
       <c r="B91" s="10"/>
       <c r="C91" s="10"/>
       <c r="F91" s="60" t="s">
-        <v>103</v>
+        <v>105</v>
       </c>
       <c r="G91" s="61">
         <f>MAX(G83-G89, 0)</f>
@@ -7007,7 +7159,7 @@
     </row>
     <row r="92" spans="2:8">
       <c r="B92" s="3" t="s">
-        <v>104</v>
+        <v>106</v>
       </c>
       <c r="C92" s="18">
         <f>C89 + C90</f>
@@ -7023,7 +7175,7 @@
     </row>
     <row r="93" spans="2:8">
       <c r="F93" t="s">
-        <v>77</v>
+        <v>79</v>
       </c>
       <c r="G93" s="6">
         <f>_xlfn.XLOOKUP(TRUE, AlternativeMinimumTaxRateTable[IsSelected], AlternativeMinimumTaxRateTable[AMT Rate], NotFoundLabelCell)</f>
@@ -7050,7 +7202,7 @@
     </row>
     <row r="94" spans="2:8">
       <c r="B94" s="56" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="C94" s="57">
         <f xml:space="preserve"> C92 / C78</f>
@@ -7064,7 +7216,7 @@
         <v>= C92 / C78</v>
       </c>
       <c r="F94" t="s">
-        <v>79</v>
+        <v>81</v>
       </c>
       <c r="G94" s="2">
         <f>_xlfn.XLOOKUP(TRUE, AlternativeMinimumTaxRateTable[IsSelected], AlternativeMinimumTaxRateTable[RangeStart], NotFoundLabelCell)</f>
@@ -7091,7 +7243,7 @@
     </row>
     <row r="95" spans="2:8">
       <c r="B95" s="56" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="C95" s="57">
         <f xml:space="preserve"> C92 / C84</f>
@@ -7107,7 +7259,7 @@
     </row>
     <row r="96" spans="2:8">
       <c r="F96" t="s">
-        <v>83</v>
+        <v>85</v>
       </c>
       <c r="G96" s="2">
         <f>IF(
@@ -7138,7 +7290,7 @@
     </row>
     <row r="97" spans="2:8">
       <c r="F97" t="s">
-        <v>85</v>
+        <v>87</v>
       </c>
       <c r="G97" s="2">
         <f xml:space="preserve"> IF(
@@ -7155,7 +7307,7 @@
     </row>
     <row r="99" spans="2:8">
       <c r="F99" s="3" t="s">
-        <v>107</v>
+        <v>109</v>
       </c>
       <c r="G99" s="18">
         <f>G96 + G97</f>
@@ -7171,7 +7323,7 @@
     </row>
     <row r="101" spans="2:8">
       <c r="F101" s="56" t="s">
-        <v>105</v>
+        <v>107</v>
       </c>
       <c r="G101" s="57">
         <f xml:space="preserve"> G99 / G78</f>
@@ -7187,7 +7339,7 @@
     </row>
     <row r="102" spans="2:8">
       <c r="F102" s="56" t="s">
-        <v>106</v>
+        <v>108</v>
       </c>
       <c r="G102" s="57">
         <f xml:space="preserve"> G99 / G83</f>
@@ -7203,7 +7355,7 @@
     </row>
     <row r="103" spans="2:8" ht="15" thickBot="1">
       <c r="B103" s="37" t="s">
-        <v>108</v>
+        <v>110</v>
       </c>
       <c r="C103" s="37"/>
     </row>
@@ -7229,7 +7381,7 @@
     </row>
     <row r="107" spans="2:8">
       <c r="B107" s="52" t="s">
-        <v>109</v>
+        <v>111</v>
       </c>
       <c r="C107" s="53">
         <f xml:space="preserve"> C84</f>
@@ -7248,7 +7400,7 @@
     </row>
     <row r="108" spans="2:8">
       <c r="B108" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C108" s="6">
         <f>_xlfn.XLOOKUP(TRUE, LongTermCapitalGainsTaxRateTable[IsBracketStart], LongTermCapitalGainsTaxRateTable[LTCG Rate], NotFoundLabelCell)</f>
@@ -7275,7 +7427,7 @@
     </row>
     <row r="109" spans="2:8">
       <c r="B109" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C109" s="2">
         <f>_xlfn.XLOOKUP(TRUE, LongTermCapitalGainsTaxRateTable[IsBracketStart], LongTermCapitalGainsTaxRateTable[RangeStart], NotFoundLabelCell)</f>
@@ -7302,7 +7454,7 @@
     </row>
     <row r="110" spans="2:8">
       <c r="B110" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C110" s="2">
         <f>IF(
@@ -7333,7 +7485,7 @@
     </row>
     <row r="111" spans="2:8">
       <c r="B111" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C111" s="2">
         <f xml:space="preserve"> IF(
@@ -7346,7 +7498,7 @@
     </row>
     <row r="112" spans="2:8">
       <c r="B112" s="62" t="s">
-        <v>114</v>
+        <v>116</v>
       </c>
       <c r="C112" s="63">
         <f xml:space="preserve"> C110 + C111</f>
@@ -7362,7 +7514,7 @@
     </row>
     <row r="114" spans="2:4">
       <c r="B114" s="52" t="s">
-        <v>115</v>
+        <v>117</v>
       </c>
       <c r="C114" s="53">
         <f xml:space="preserve"> C107 + C105</f>
@@ -7378,7 +7530,7 @@
     </row>
     <row r="115" spans="2:4">
       <c r="B115" t="s">
-        <v>110</v>
+        <v>112</v>
       </c>
       <c r="C115" s="6">
         <f>_xlfn.XLOOKUP(TRUE, LongTermCapitalGainsTaxRateTable[IsBracketEnd], LongTermCapitalGainsTaxRateTable[LTCG Rate], NotFoundLabelCell)</f>
@@ -7405,7 +7557,7 @@
     </row>
     <row r="116" spans="2:4">
       <c r="B116" t="s">
-        <v>111</v>
+        <v>113</v>
       </c>
       <c r="C116" s="2">
         <f>_xlfn.XLOOKUP(TRUE, LongTermCapitalGainsTaxRateTable[IsBracketEnd], LongTermCapitalGainsTaxRateTable[RangeStart], NotFoundLabelCell)</f>
@@ -7432,7 +7584,7 @@
     </row>
     <row r="117" spans="2:4">
       <c r="B117" t="s">
-        <v>112</v>
+        <v>114</v>
       </c>
       <c r="C117" s="2">
         <f>IF(
@@ -7463,7 +7615,7 @@
     </row>
     <row r="118" spans="2:4">
       <c r="B118" t="s">
-        <v>113</v>
+        <v>115</v>
       </c>
       <c r="C118" s="2">
         <f xml:space="preserve"> IF(
@@ -7476,7 +7628,7 @@
     </row>
     <row r="119" spans="2:4">
       <c r="B119" s="62" t="s">
-        <v>116</v>
+        <v>118</v>
       </c>
       <c r="C119" s="63">
         <f xml:space="preserve"> C117 + C118</f>
@@ -7496,7 +7648,7 @@
     </row>
     <row r="121" spans="2:4">
       <c r="B121" s="3" t="s">
-        <v>117</v>
+        <v>119</v>
       </c>
       <c r="C121" s="4">
         <f xml:space="preserve"> C119 - C112</f>
@@ -7512,7 +7664,7 @@
     </row>
     <row r="123" spans="2:4">
       <c r="B123" s="56" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C123" s="57">
         <f xml:space="preserve"> C121 / C105</f>
@@ -7612,7 +7764,7 @@
   <sheetData>
     <row r="2" spans="2:12" ht="15.6">
       <c r="B2" s="23" t="s">
-        <v>119</v>
+        <v>121</v>
       </c>
       <c r="C2" s="23"/>
       <c r="D2" s="23"/>
@@ -7623,7 +7775,7 @@
     </row>
     <row r="3" spans="2:12" ht="15.6">
       <c r="B3" s="23" t="s">
-        <v>120</v>
+        <v>122</v>
       </c>
       <c r="C3" s="23"/>
       <c r="D3" s="23"/>
@@ -7641,17 +7793,17 @@
         <v>FilingStatusTable</v>
       </c>
       <c r="C6" s="13" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D6" s="14" t="str">
         <f>FilingStatusTable[[#Headers],[Filing Status]]</f>
         <v>Filing Status</v>
       </c>
       <c r="F6" t="s">
-        <v>122</v>
+        <v>124</v>
       </c>
       <c r="G6" s="21" t="s">
-        <v>123</v>
+        <v>125</v>
       </c>
     </row>
     <row r="7" spans="2:12">
@@ -7663,51 +7815,51 @@
         <v>Valid</v>
       </c>
       <c r="F7" t="s">
-        <v>124</v>
+        <v>126</v>
       </c>
       <c r="G7" s="21" t="s">
-        <v>125</v>
+        <v>127</v>
       </c>
     </row>
     <row r="8" spans="2:12">
       <c r="B8" s="24" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="C8" s="24" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="F8" t="s">
-        <v>128</v>
+        <v>130</v>
       </c>
       <c r="G8" s="21" t="s">
-        <v>129</v>
+        <v>131</v>
       </c>
     </row>
     <row r="9" spans="2:12">
       <c r="B9" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="C9" t="b">
         <f xml:space="preserve"> (FilingStatusTable[[#This Row],[Filing Status]] = EstimateInputFilingStatusCell)</f>
         <v>1</v>
       </c>
       <c r="F9" t="s">
-        <v>130</v>
+        <v>132</v>
       </c>
       <c r="G9" s="21" t="s">
-        <v>131</v>
+        <v>133</v>
       </c>
     </row>
     <row r="10" spans="2:12" ht="15">
       <c r="B10" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="C10" t="b">
         <f xml:space="preserve"> (FilingStatusTable[[#This Row],[Filing Status]] = EstimateInputFilingStatusCell)</f>
         <v>0</v>
       </c>
       <c r="F10" t="s">
-        <v>133</v>
+        <v>135</v>
       </c>
       <c r="G10" s="79">
         <v>10000000</v>
@@ -7715,7 +7867,7 @@
     </row>
     <row r="11" spans="2:12">
       <c r="B11" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="C11" t="b">
         <f xml:space="preserve"> (FilingStatusTable[[#This Row],[Filing Status]] = EstimateInputFilingStatusCell)</f>
@@ -7724,7 +7876,7 @@
     </row>
     <row r="12" spans="2:12">
       <c r="B12" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="C12" t="b">
         <f xml:space="preserve"> (FilingStatusTable[[#This Row],[Filing Status]] = EstimateInputFilingStatusCell)</f>
@@ -7740,7 +7892,7 @@
         <v>MedicareWageTaxRateTable</v>
       </c>
       <c r="G14" s="13" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="H14" s="14" t="str">
         <f>MedicareWageTaxRateTable[[#Headers],[Medicare Rate]]</f>
@@ -7765,32 +7917,32 @@
         <v>SupportedYearsTable</v>
       </c>
       <c r="C16" s="13" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="D16" s="14" t="str">
         <f>SupportedYearsTable[[#Headers],[Tax Year]]</f>
         <v>Tax Year</v>
       </c>
       <c r="F16" s="24" t="s">
-        <v>126</v>
+        <v>128</v>
       </c>
       <c r="G16" s="24" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="H16" s="24" t="s">
-        <v>137</v>
+        <v>139</v>
       </c>
       <c r="I16" s="24" t="s">
-        <v>138</v>
+        <v>140</v>
       </c>
       <c r="J16" s="24" t="s">
-        <v>139</v>
+        <v>141</v>
       </c>
       <c r="K16" s="24" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="L16" s="24" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="17" spans="2:12">
@@ -7802,7 +7954,7 @@
         <v>Valid</v>
       </c>
       <c r="F17" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G17" s="7">
         <v>2024</v>
@@ -7831,13 +7983,13 @@
     </row>
     <row r="18" spans="2:12">
       <c r="B18" s="24" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="C18" s="24" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
       <c r="F18" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G18" s="7">
         <v>2024</v>
@@ -7877,7 +8029,7 @@
         <v>0</v>
       </c>
       <c r="F19" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G19" s="7">
         <v>2024</v>
@@ -7913,7 +8065,7 @@
         <v>1</v>
       </c>
       <c r="F20" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G20" s="7">
         <v>2024</v>
@@ -7946,7 +8098,7 @@
     </row>
     <row r="21" spans="2:12">
       <c r="F21" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G21" s="7">
         <v>2024</v>
@@ -7975,7 +8127,7 @@
     </row>
     <row r="22" spans="2:12">
       <c r="F22" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G22" s="7">
         <v>2024</v>
@@ -8008,7 +8160,7 @@
     </row>
     <row r="23" spans="2:12">
       <c r="F23" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G23" s="7">
         <v>2024</v>
@@ -8037,7 +8189,7 @@
     </row>
     <row r="24" spans="2:12">
       <c r="F24" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G24" s="7">
         <v>2024</v>
@@ -8087,7 +8239,7 @@
     </row>
     <row r="26" spans="2:12">
       <c r="F26" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G26" s="7">
         <v>2025</v>
@@ -8116,7 +8268,7 @@
     </row>
     <row r="27" spans="2:12">
       <c r="F27" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G27" s="7">
         <v>2025</v>
@@ -8149,7 +8301,7 @@
     </row>
     <row r="28" spans="2:12">
       <c r="F28" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G28" s="7">
         <v>2025</v>
@@ -8178,7 +8330,7 @@
     </row>
     <row r="29" spans="2:12">
       <c r="F29" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G29" s="7">
         <v>2025</v>
@@ -8211,7 +8363,7 @@
     </row>
     <row r="30" spans="2:12">
       <c r="F30" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G30" s="7">
         <v>2025</v>
@@ -8240,7 +8392,7 @@
     </row>
     <row r="31" spans="2:12">
       <c r="F31" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G31" s="7">
         <v>2025</v>
@@ -8273,7 +8425,7 @@
     </row>
     <row r="32" spans="2:12">
       <c r="F32" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G32" s="7">
         <v>2025</v>
@@ -8302,7 +8454,7 @@
     </row>
     <row r="33" spans="6:12">
       <c r="F33" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G33" s="7">
         <v>2025</v>
@@ -8342,7 +8494,7 @@
         <v>MedicareNetInvestIncomeTaxTable</v>
       </c>
       <c r="G37" s="13" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="H37" s="14" t="str">
         <f>MedicareNetInvestIncomeTaxTable[[#Headers],[NetInvestInc Rate]]</f>
@@ -8360,24 +8512,24 @@
     </row>
     <row r="39" spans="6:12">
       <c r="F39" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="G39" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="H39" t="s">
-        <v>142</v>
+        <v>144</v>
       </c>
       <c r="I39" t="s">
-        <v>143</v>
+        <v>145</v>
       </c>
       <c r="J39" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="40" spans="6:12">
       <c r="F40" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G40" s="7">
         <v>2024</v>
@@ -8398,7 +8550,7 @@
     </row>
     <row r="41" spans="6:12">
       <c r="F41" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G41" s="7">
         <v>2024</v>
@@ -8419,7 +8571,7 @@
     </row>
     <row r="42" spans="6:12">
       <c r="F42" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G42" s="7">
         <v>2024</v>
@@ -8440,7 +8592,7 @@
     </row>
     <row r="43" spans="6:12">
       <c r="F43" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G43" s="7">
         <v>2024</v>
@@ -8474,7 +8626,7 @@
     </row>
     <row r="45" spans="6:12">
       <c r="F45" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G45" s="7">
         <v>2025</v>
@@ -8495,7 +8647,7 @@
     </row>
     <row r="46" spans="6:12">
       <c r="F46" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G46" s="7">
         <v>2025</v>
@@ -8516,7 +8668,7 @@
     </row>
     <row r="47" spans="6:12">
       <c r="F47" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G47" s="7">
         <v>2025</v>
@@ -8537,7 +8689,7 @@
     </row>
     <row r="48" spans="6:12">
       <c r="F48" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G48" s="7">
         <v>2025</v>
@@ -8565,7 +8717,7 @@
         <v>SocialSecurityTaxRateTable</v>
       </c>
       <c r="G52" s="13" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="H52" s="14" t="str">
         <f>SocialSecurityTaxRateTable[[#Headers],[SocialSecurity Rate]]</f>
@@ -8583,27 +8735,27 @@
     </row>
     <row r="54" spans="6:11">
       <c r="F54" s="24" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="G54" s="24" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="H54" s="24" t="s">
-        <v>144</v>
+        <v>146</v>
       </c>
       <c r="I54" s="24" t="s">
-        <v>145</v>
+        <v>147</v>
       </c>
       <c r="J54" s="24" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="K54" s="24" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="55" spans="6:11">
       <c r="F55" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G55" s="7">
         <v>2024</v>
@@ -8627,7 +8779,7 @@
     </row>
     <row r="56" spans="6:11">
       <c r="F56" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G56" s="7">
         <v>2024</v>
@@ -8651,7 +8803,7 @@
     </row>
     <row r="57" spans="6:11">
       <c r="F57" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G57" s="7">
         <v>2024</v>
@@ -8675,7 +8827,7 @@
     </row>
     <row r="58" spans="6:11">
       <c r="F58" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G58" s="7">
         <v>2024</v>
@@ -8713,7 +8865,7 @@
     </row>
     <row r="60" spans="6:11">
       <c r="F60" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G60" s="7">
         <v>2025</v>
@@ -8737,7 +8889,7 @@
     </row>
     <row r="61" spans="6:11">
       <c r="F61" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G61" s="7">
         <v>2025</v>
@@ -8761,7 +8913,7 @@
     </row>
     <row r="62" spans="6:11">
       <c r="F62" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G62" s="7">
         <v>2025</v>
@@ -8785,7 +8937,7 @@
     </row>
     <row r="63" spans="6:11">
       <c r="F63" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G63" s="7">
         <v>2025</v>
@@ -8816,7 +8968,7 @@
         <v>StandardDeductionAmountTable</v>
       </c>
       <c r="G67" s="13" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="H67" s="14" t="str">
         <f>StandardDeductionAmountTable[[#Headers],[Standard 
@@ -8836,21 +8988,21 @@
     </row>
     <row r="69" spans="6:9" ht="27.6">
       <c r="F69" s="44" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="G69" s="44" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="H69" s="45" t="s">
-        <v>146</v>
+        <v>148</v>
       </c>
       <c r="I69" s="44" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="70" spans="6:9">
       <c r="F70" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G70" s="7">
         <v>2024</v>
@@ -8868,7 +9020,7 @@
     </row>
     <row r="71" spans="6:9">
       <c r="F71" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G71" s="7">
         <v>2024</v>
@@ -8886,7 +9038,7 @@
     </row>
     <row r="72" spans="6:9">
       <c r="F72" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G72" s="7">
         <v>2024</v>
@@ -8904,7 +9056,7 @@
     </row>
     <row r="73" spans="6:9">
       <c r="F73" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G73" s="7">
         <v>2024</v>
@@ -8934,7 +9086,7 @@
     </row>
     <row r="75" spans="6:9">
       <c r="F75" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G75" s="7">
         <v>2025</v>
@@ -8952,7 +9104,7 @@
     </row>
     <row r="76" spans="6:9">
       <c r="F76" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G76" s="7">
         <v>2025</v>
@@ -8970,7 +9122,7 @@
     </row>
     <row r="77" spans="6:9">
       <c r="F77" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G77" s="7">
         <v>2025</v>
@@ -8988,7 +9140,7 @@
     </row>
     <row r="78" spans="6:9">
       <c r="F78" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G78" s="7">
         <v>2025</v>
@@ -9013,7 +9165,7 @@
         <v>FederalIncomeTaxRateTable</v>
       </c>
       <c r="G82" s="13" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="H82" s="14" t="str">
         <f>FederalIncomeTaxRateTable[[#Headers],[Federal Tax Rate]]</f>
@@ -9031,30 +9183,30 @@
     </row>
     <row r="84" spans="6:12">
       <c r="F84" s="24" t="s">
+        <v>143</v>
+      </c>
+      <c r="G84" s="24" t="s">
+        <v>138</v>
+      </c>
+      <c r="H84" s="24" t="s">
+        <v>149</v>
+      </c>
+      <c r="I84" s="24" t="s">
+        <v>140</v>
+      </c>
+      <c r="J84" s="24" t="s">
         <v>141</v>
       </c>
-      <c r="G84" s="24" t="s">
-        <v>136</v>
-      </c>
-      <c r="H84" s="24" t="s">
-        <v>147</v>
-      </c>
-      <c r="I84" s="24" t="s">
-        <v>138</v>
-      </c>
-      <c r="J84" s="24" t="s">
-        <v>139</v>
-      </c>
       <c r="K84" s="24" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="L84" s="24" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="85" spans="6:12">
       <c r="F85" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G85" s="7">
         <v>2024</v>
@@ -9083,7 +9235,7 @@
     </row>
     <row r="86" spans="6:12">
       <c r="F86" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G86" s="7">
         <v>2024</v>
@@ -9114,7 +9266,7 @@
     </row>
     <row r="87" spans="6:12">
       <c r="F87" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G87" s="7">
         <v>2024</v>
@@ -9145,7 +9297,7 @@
     </row>
     <row r="88" spans="6:12">
       <c r="F88" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G88" s="7">
         <v>2024</v>
@@ -9176,7 +9328,7 @@
     </row>
     <row r="89" spans="6:12">
       <c r="F89" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G89" s="7">
         <v>2024</v>
@@ -9207,7 +9359,7 @@
     </row>
     <row r="90" spans="6:12">
       <c r="F90" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G90" s="7">
         <v>2024</v>
@@ -9238,7 +9390,7 @@
     </row>
     <row r="91" spans="6:12">
       <c r="F91" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G91" s="7">
         <v>2024</v>
@@ -9270,7 +9422,7 @@
     </row>
     <row r="92" spans="6:12">
       <c r="F92" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G92" s="7">
         <v>2024</v>
@@ -9299,7 +9451,7 @@
     </row>
     <row r="93" spans="6:12">
       <c r="F93" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G93" s="7">
         <v>2024</v>
@@ -9330,7 +9482,7 @@
     </row>
     <row r="94" spans="6:12">
       <c r="F94" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G94" s="7">
         <v>2024</v>
@@ -9361,7 +9513,7 @@
     </row>
     <row r="95" spans="6:12">
       <c r="F95" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G95" s="7">
         <v>2024</v>
@@ -9392,7 +9544,7 @@
     </row>
     <row r="96" spans="6:12">
       <c r="F96" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G96" s="7">
         <v>2024</v>
@@ -9423,7 +9575,7 @@
     </row>
     <row r="97" spans="6:12">
       <c r="F97" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G97" s="7">
         <v>2024</v>
@@ -9454,7 +9606,7 @@
     </row>
     <row r="98" spans="6:12">
       <c r="F98" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G98" s="7">
         <v>2024</v>
@@ -9486,7 +9638,7 @@
     </row>
     <row r="99" spans="6:12">
       <c r="F99" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G99" s="7">
         <v>2024</v>
@@ -9515,7 +9667,7 @@
     </row>
     <row r="100" spans="6:12">
       <c r="F100" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G100" s="7">
         <v>2024</v>
@@ -9546,7 +9698,7 @@
     </row>
     <row r="101" spans="6:12">
       <c r="F101" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G101" s="7">
         <v>2024</v>
@@ -9577,7 +9729,7 @@
     </row>
     <row r="102" spans="6:12">
       <c r="F102" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G102" s="7">
         <v>2024</v>
@@ -9608,7 +9760,7 @@
     </row>
     <row r="103" spans="6:12">
       <c r="F103" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G103" s="7">
         <v>2024</v>
@@ -9639,7 +9791,7 @@
     </row>
     <row r="104" spans="6:12">
       <c r="F104" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G104" s="7">
         <v>2024</v>
@@ -9670,7 +9822,7 @@
     </row>
     <row r="105" spans="6:12">
       <c r="F105" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G105" s="7">
         <v>2024</v>
@@ -9702,7 +9854,7 @@
     </row>
     <row r="106" spans="6:12">
       <c r="F106" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G106" s="7">
         <v>2024</v>
@@ -9731,7 +9883,7 @@
     </row>
     <row r="107" spans="6:12">
       <c r="F107" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G107" s="7">
         <v>2024</v>
@@ -9762,7 +9914,7 @@
     </row>
     <row r="108" spans="6:12">
       <c r="F108" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G108" s="7">
         <v>2024</v>
@@ -9793,7 +9945,7 @@
     </row>
     <row r="109" spans="6:12">
       <c r="F109" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G109" s="7">
         <v>2024</v>
@@ -9824,7 +9976,7 @@
     </row>
     <row r="110" spans="6:12">
       <c r="F110" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G110" s="7">
         <v>2024</v>
@@ -9855,7 +10007,7 @@
     </row>
     <row r="111" spans="6:12">
       <c r="F111" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G111" s="7">
         <v>2024</v>
@@ -9886,7 +10038,7 @@
     </row>
     <row r="112" spans="6:12">
       <c r="F112" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G112" s="7">
         <v>2024</v>
@@ -9934,7 +10086,7 @@
     </row>
     <row r="114" spans="6:12">
       <c r="F114" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G114" s="7">
         <v>2025</v>
@@ -9963,7 +10115,7 @@
     </row>
     <row r="115" spans="6:12">
       <c r="F115" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G115" s="7">
         <v>2025</v>
@@ -9994,7 +10146,7 @@
     </row>
     <row r="116" spans="6:12">
       <c r="F116" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G116" s="7">
         <v>2025</v>
@@ -10025,7 +10177,7 @@
     </row>
     <row r="117" spans="6:12">
       <c r="F117" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G117" s="7">
         <v>2025</v>
@@ -10056,7 +10208,7 @@
     </row>
     <row r="118" spans="6:12">
       <c r="F118" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G118" s="7">
         <v>2025</v>
@@ -10087,7 +10239,7 @@
     </row>
     <row r="119" spans="6:12">
       <c r="F119" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G119" s="7">
         <v>2025</v>
@@ -10118,7 +10270,7 @@
     </row>
     <row r="120" spans="6:12">
       <c r="F120" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G120" s="7">
         <v>2025</v>
@@ -10150,7 +10302,7 @@
     </row>
     <row r="121" spans="6:12">
       <c r="F121" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G121" s="7">
         <v>2025</v>
@@ -10179,7 +10331,7 @@
     </row>
     <row r="122" spans="6:12">
       <c r="F122" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G122" s="7">
         <v>2025</v>
@@ -10210,7 +10362,7 @@
     </row>
     <row r="123" spans="6:12">
       <c r="F123" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G123" s="7">
         <v>2025</v>
@@ -10241,7 +10393,7 @@
     </row>
     <row r="124" spans="6:12">
       <c r="F124" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G124" s="7">
         <v>2025</v>
@@ -10272,7 +10424,7 @@
     </row>
     <row r="125" spans="6:12">
       <c r="F125" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G125" s="7">
         <v>2025</v>
@@ -10303,7 +10455,7 @@
     </row>
     <row r="126" spans="6:12">
       <c r="F126" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G126" s="7">
         <v>2025</v>
@@ -10334,7 +10486,7 @@
     </row>
     <row r="127" spans="6:12">
       <c r="F127" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G127" s="7">
         <v>2025</v>
@@ -10366,7 +10518,7 @@
     </row>
     <row r="128" spans="6:12">
       <c r="F128" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G128" s="7">
         <v>2025</v>
@@ -10395,7 +10547,7 @@
     </row>
     <row r="129" spans="6:12">
       <c r="F129" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G129" s="7">
         <v>2025</v>
@@ -10426,7 +10578,7 @@
     </row>
     <row r="130" spans="6:12">
       <c r="F130" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G130" s="7">
         <v>2025</v>
@@ -10457,7 +10609,7 @@
     </row>
     <row r="131" spans="6:12">
       <c r="F131" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G131" s="7">
         <v>2025</v>
@@ -10488,7 +10640,7 @@
     </row>
     <row r="132" spans="6:12">
       <c r="F132" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G132" s="7">
         <v>2025</v>
@@ -10519,7 +10671,7 @@
     </row>
     <row r="133" spans="6:12">
       <c r="F133" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G133" s="7">
         <v>2025</v>
@@ -10550,7 +10702,7 @@
     </row>
     <row r="134" spans="6:12">
       <c r="F134" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G134" s="7">
         <v>2025</v>
@@ -10582,7 +10734,7 @@
     </row>
     <row r="135" spans="6:12">
       <c r="F135" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G135" s="7">
         <v>2025</v>
@@ -10611,7 +10763,7 @@
     </row>
     <row r="136" spans="6:12">
       <c r="F136" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G136" s="7">
         <v>2025</v>
@@ -10642,7 +10794,7 @@
     </row>
     <row r="137" spans="6:12">
       <c r="F137" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G137" s="7">
         <v>2025</v>
@@ -10673,7 +10825,7 @@
     </row>
     <row r="138" spans="6:12">
       <c r="F138" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G138" s="7">
         <v>2025</v>
@@ -10704,7 +10856,7 @@
     </row>
     <row r="139" spans="6:12">
       <c r="F139" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G139" s="7">
         <v>2025</v>
@@ -10735,7 +10887,7 @@
     </row>
     <row r="140" spans="6:12">
       <c r="F140" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G140" s="7">
         <v>2025</v>
@@ -10766,7 +10918,7 @@
     </row>
     <row r="141" spans="6:12">
       <c r="F141" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G141" s="7">
         <v>2025</v>
@@ -10805,7 +10957,7 @@
         <v>AlternativeMimumumTaxThresholdsTable</v>
       </c>
       <c r="G145" s="13" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="H145" s="14" t="str">
         <f>AlternativeMimumumTaxThresholdsTable[[#Headers],[AMT Exemption]]</f>
@@ -10823,24 +10975,24 @@
     </row>
     <row r="147" spans="6:10">
       <c r="F147" t="s">
-        <v>141</v>
+        <v>143</v>
       </c>
       <c r="G147" t="s">
-        <v>136</v>
+        <v>138</v>
       </c>
       <c r="H147" t="s">
-        <v>148</v>
+        <v>150</v>
       </c>
       <c r="I147" t="s">
-        <v>149</v>
+        <v>151</v>
       </c>
       <c r="J147" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="148" spans="6:10">
       <c r="F148" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G148" s="7">
         <v>2024</v>
@@ -10861,7 +11013,7 @@
     </row>
     <row r="149" spans="6:10">
       <c r="F149" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G149" s="7">
         <v>2024</v>
@@ -10882,7 +11034,7 @@
     </row>
     <row r="150" spans="6:10">
       <c r="F150" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G150" s="7">
         <v>2024</v>
@@ -10903,7 +11055,7 @@
     </row>
     <row r="151" spans="6:10">
       <c r="F151" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G151" s="7">
         <v>2024</v>
@@ -10937,7 +11089,7 @@
     </row>
     <row r="153" spans="6:10">
       <c r="F153" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G153" s="7">
         <v>2025</v>
@@ -10958,7 +11110,7 @@
     </row>
     <row r="154" spans="6:10">
       <c r="F154" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G154" s="7">
         <v>2025</v>
@@ -10979,7 +11131,7 @@
     </row>
     <row r="155" spans="6:10">
       <c r="F155" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G155" s="7">
         <v>2025</v>
@@ -11000,7 +11152,7 @@
     </row>
     <row r="156" spans="6:10">
       <c r="F156" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G156" s="7">
         <v>2025</v>
@@ -11028,7 +11180,7 @@
         <v>AlternativeMinimumTaxRateTable</v>
       </c>
       <c r="G160" s="13" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="H160" s="14" t="str">
         <f>AlternativeMinimumTaxRateTable[[#Headers],[AMT Rate]]</f>
@@ -11046,30 +11198,30 @@
     </row>
     <row r="162" spans="6:12">
       <c r="F162" s="24" t="s">
+        <v>143</v>
+      </c>
+      <c r="G162" s="24" t="s">
+        <v>138</v>
+      </c>
+      <c r="H162" s="24" t="s">
+        <v>152</v>
+      </c>
+      <c r="I162" s="24" t="s">
+        <v>140</v>
+      </c>
+      <c r="J162" s="24" t="s">
         <v>141</v>
       </c>
-      <c r="G162" s="24" t="s">
-        <v>136</v>
-      </c>
-      <c r="H162" s="24" t="s">
-        <v>150</v>
-      </c>
-      <c r="I162" s="24" t="s">
-        <v>138</v>
-      </c>
-      <c r="J162" s="24" t="s">
-        <v>139</v>
-      </c>
       <c r="K162" s="24" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="L162" s="24" t="s">
-        <v>127</v>
+        <v>129</v>
       </c>
     </row>
     <row r="163" spans="6:12">
       <c r="F163" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G163" s="7">
         <v>2024</v>
@@ -11098,7 +11250,7 @@
     </row>
     <row r="164" spans="6:12">
       <c r="F164" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G164" s="7">
         <v>2024</v>
@@ -11130,7 +11282,7 @@
     </row>
     <row r="165" spans="6:12">
       <c r="F165" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G165" s="7">
         <v>2024</v>
@@ -11159,7 +11311,7 @@
     </row>
     <row r="166" spans="6:12">
       <c r="F166" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G166" s="7">
         <v>2024</v>
@@ -11191,7 +11343,7 @@
     </row>
     <row r="167" spans="6:12">
       <c r="F167" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G167" s="7">
         <v>2024</v>
@@ -11220,7 +11372,7 @@
     </row>
     <row r="168" spans="6:12">
       <c r="F168" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G168" s="7">
         <v>2024</v>
@@ -11252,7 +11404,7 @@
     </row>
     <row r="169" spans="6:12">
       <c r="F169" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G169" s="7">
         <v>2024</v>
@@ -11281,7 +11433,7 @@
     </row>
     <row r="170" spans="6:12">
       <c r="F170" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G170" s="7">
         <v>2024</v>
@@ -11330,7 +11482,7 @@
     </row>
     <row r="172" spans="6:12">
       <c r="F172" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G172" s="7">
         <v>2025</v>
@@ -11359,7 +11511,7 @@
     </row>
     <row r="173" spans="6:12">
       <c r="F173" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G173" s="7">
         <v>2025</v>
@@ -11391,7 +11543,7 @@
     </row>
     <row r="174" spans="6:12">
       <c r="F174" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G174" s="7">
         <v>2025</v>
@@ -11420,7 +11572,7 @@
     </row>
     <row r="175" spans="6:12">
       <c r="F175" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G175" s="7">
         <v>2025</v>
@@ -11452,7 +11604,7 @@
     </row>
     <row r="176" spans="6:12">
       <c r="F176" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G176" s="7">
         <v>2025</v>
@@ -11481,7 +11633,7 @@
     </row>
     <row r="177" spans="6:13">
       <c r="F177" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G177" s="7">
         <v>2025</v>
@@ -11513,7 +11665,7 @@
     </row>
     <row r="178" spans="6:13">
       <c r="F178" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G178" s="7">
         <v>2025</v>
@@ -11542,7 +11694,7 @@
     </row>
     <row r="179" spans="6:13">
       <c r="F179" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G179" s="7">
         <v>2025</v>
@@ -11581,7 +11733,7 @@
         <v>LongTermCapitalGainsTaxRateTable</v>
       </c>
       <c r="G183" s="13" t="s">
-        <v>121</v>
+        <v>123</v>
       </c>
       <c r="H183" s="14" t="str">
         <f>LongTermCapitalGainsTaxRateTable[[#Headers],[LTCG Rate]]</f>
@@ -11606,33 +11758,33 @@
     </row>
     <row r="185" spans="6:13">
       <c r="F185" s="24" t="s">
+        <v>143</v>
+      </c>
+      <c r="G185" s="24" t="s">
+        <v>138</v>
+      </c>
+      <c r="H185" s="24" t="s">
+        <v>153</v>
+      </c>
+      <c r="I185" s="24" t="s">
+        <v>140</v>
+      </c>
+      <c r="J185" s="24" t="s">
         <v>141</v>
       </c>
-      <c r="G185" s="24" t="s">
-        <v>136</v>
-      </c>
-      <c r="H185" s="24" t="s">
-        <v>151</v>
-      </c>
-      <c r="I185" s="24" t="s">
-        <v>138</v>
-      </c>
-      <c r="J185" s="24" t="s">
-        <v>139</v>
-      </c>
       <c r="K185" s="24" t="s">
-        <v>140</v>
+        <v>142</v>
       </c>
       <c r="L185" s="24" t="s">
-        <v>152</v>
+        <v>154</v>
       </c>
       <c r="M185" s="24" t="s">
-        <v>153</v>
+        <v>155</v>
       </c>
     </row>
     <row r="186" spans="6:13">
       <c r="F186" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G186" s="7">
         <v>2024</v>
@@ -11670,7 +11822,7 @@
     </row>
     <row r="187" spans="6:13">
       <c r="F187" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G187" s="7">
         <v>2024</v>
@@ -11710,7 +11862,7 @@
     </row>
     <row r="188" spans="6:13">
       <c r="F188" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G188" s="7">
         <v>2024</v>
@@ -11751,7 +11903,7 @@
     </row>
     <row r="189" spans="6:13">
       <c r="F189" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G189" s="7">
         <v>2024</v>
@@ -11789,7 +11941,7 @@
     </row>
     <row r="190" spans="6:13">
       <c r="F190" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G190" s="7">
         <v>2024</v>
@@ -11829,7 +11981,7 @@
     </row>
     <row r="191" spans="6:13">
       <c r="F191" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G191" s="7">
         <v>2024</v>
@@ -11870,7 +12022,7 @@
     </row>
     <row r="192" spans="6:13">
       <c r="F192" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G192" s="7">
         <v>2024</v>
@@ -11908,7 +12060,7 @@
     </row>
     <row r="193" spans="6:13">
       <c r="F193" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G193" s="7">
         <v>2024</v>
@@ -11948,7 +12100,7 @@
     </row>
     <row r="194" spans="6:13">
       <c r="F194" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G194" s="7">
         <v>2024</v>
@@ -11989,7 +12141,7 @@
     </row>
     <row r="195" spans="6:13">
       <c r="F195" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G195" s="7">
         <v>2024</v>
@@ -12027,7 +12179,7 @@
     </row>
     <row r="196" spans="6:13">
       <c r="F196" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G196" s="7">
         <v>2024</v>
@@ -12067,7 +12219,7 @@
     </row>
     <row r="197" spans="6:13">
       <c r="F197" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G197" s="7">
         <v>2024</v>
@@ -12133,7 +12285,7 @@
     </row>
     <row r="199" spans="6:13">
       <c r="F199" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G199" s="7">
         <v>2025</v>
@@ -12171,7 +12323,7 @@
     </row>
     <row r="200" spans="6:13">
       <c r="F200" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G200" s="7">
         <v>2025</v>
@@ -12211,7 +12363,7 @@
     </row>
     <row r="201" spans="6:13">
       <c r="F201" s="6" t="s">
-        <v>16</v>
+        <v>18</v>
       </c>
       <c r="G201" s="7">
         <v>2025</v>
@@ -12252,7 +12404,7 @@
     </row>
     <row r="202" spans="6:13">
       <c r="F202" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G202" s="7">
         <v>2025</v>
@@ -12290,7 +12442,7 @@
     </row>
     <row r="203" spans="6:13">
       <c r="F203" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G203" s="7">
         <v>2025</v>
@@ -12330,7 +12482,7 @@
     </row>
     <row r="204" spans="6:13">
       <c r="F204" s="6" t="s">
-        <v>132</v>
+        <v>134</v>
       </c>
       <c r="G204" s="7">
         <v>2025</v>
@@ -12371,7 +12523,7 @@
     </row>
     <row r="205" spans="6:13">
       <c r="F205" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G205" s="7">
         <v>2025</v>
@@ -12409,7 +12561,7 @@
     </row>
     <row r="206" spans="6:13">
       <c r="F206" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G206" s="7">
         <v>2025</v>
@@ -12449,7 +12601,7 @@
     </row>
     <row r="207" spans="6:13">
       <c r="F207" s="6" t="s">
-        <v>134</v>
+        <v>136</v>
       </c>
       <c r="G207" s="7">
         <v>2025</v>
@@ -12490,7 +12642,7 @@
     </row>
     <row r="208" spans="6:13">
       <c r="F208" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G208" s="7">
         <v>2025</v>
@@ -12528,7 +12680,7 @@
     </row>
     <row r="209" spans="6:13">
       <c r="F209" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G209" s="7">
         <v>2025</v>
@@ -12568,7 +12720,7 @@
     </row>
     <row r="210" spans="6:13">
       <c r="F210" s="6" t="s">
-        <v>135</v>
+        <v>137</v>
       </c>
       <c r="G210" s="7">
         <v>2025</v>

</xml_diff>

<commit_message>
Fix min value for the income chart scale to 0
</commit_message>
<xml_diff>
--- a/Combined Tax Estimator.xlsx
+++ b/Combined Tax Estimator.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://d.docs.live.net/ab913e7457364688/Documents/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{F3B28514-71F1-41DD-9E29-9270D63E5505}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{AC3D1E9F-2F0D-45CF-A5F4-49429CE23319}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="18636" yWindow="492" windowWidth="26892" windowHeight="22536" xr2:uid="{F29755CA-56C7-4287-B0E1-95271A5704F5}"/>
   </bookViews>
@@ -3001,6 +3001,7 @@
         <c:axId val="1176685488"/>
         <c:scaling>
           <c:orientation val="minMax"/>
+          <c:min val="0"/>
         </c:scaling>
         <c:delete val="0"/>
         <c:axPos val="l"/>
@@ -5446,7 +5447,7 @@
   <dimension ref="B3:B17"/>
   <sheetFormatPr defaultRowHeight="14.45"/>
   <cols>
-    <col min="2" max="2" width="85" style="77" customWidth="1"/>
+    <col min="2" max="2" width="89.28515625" style="77" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="3" spans="2:2" ht="18" thickBot="1">
@@ -5464,7 +5465,7 @@
         <v>2</v>
       </c>
     </row>
-    <row r="7" spans="2:2" ht="298.5" customHeight="1" thickTop="1">
+    <row r="7" spans="2:2" ht="269.25" customHeight="1" thickTop="1">
       <c r="B7" s="81" t="s">
         <v>3</v>
       </c>

</xml_diff>

<commit_message>
Fix favicon on embed page & font for total tax
</commit_message>
<xml_diff>
--- a/Combined Tax Estimator.xlsx
+++ b/Combined Tax Estimator.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\00\Code\GitHub\Combined-Income-Tax-Estimator\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7B128771-BA47-41DC-B525-D2EF2933E66E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7A0FCBBF-AC17-4DAC-8B6C-B09D2872B321}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="2904" yWindow="0" windowWidth="35256" windowHeight="23784" activeTab="1" xr2:uid="{F29755CA-56C7-4287-B0E1-95271A5704F5}"/>
+    <workbookView xWindow="7056" yWindow="1056" windowWidth="35256" windowHeight="23784" activeTab="1" xr2:uid="{F29755CA-56C7-4287-B0E1-95271A5704F5}"/>
   </bookViews>
   <sheets>
     <sheet name="ReadMe" sheetId="3" r:id="rId1"/>
@@ -1739,7 +1739,7 @@
     <xf numFmtId="0" fontId="28" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="35" fillId="0" borderId="9" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="115">
+  <cellXfs count="116">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="1" applyNumberFormat="1" applyFont="1"/>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1"/>
@@ -1901,11 +1901,6 @@
     <xf numFmtId="0" fontId="42" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="26" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="1" xfId="3" quotePrefix="1" applyFont="1" applyAlignment="1"/>
-    <xf numFmtId="0" fontId="41" fillId="0" borderId="1" xfId="3" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="43" fillId="6" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="left"/>
     </xf>
@@ -1928,12 +1923,12 @@
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="4" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="4" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="4" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="167" fontId="4" fillId="6" borderId="14" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="46" fillId="6" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="left" vertical="center" indent="2"/>
     </xf>
-    <xf numFmtId="168" fontId="46" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="168" fontId="46" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="167" fontId="46" fillId="6" borderId="14" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
@@ -1943,14 +1938,20 @@
     <xf numFmtId="168" fontId="4" fillId="4" borderId="16" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="167" fontId="4" fillId="4" borderId="17" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="4" fillId="8" borderId="13" xfId="0" applyFont="1" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
     <xf numFmtId="167" fontId="4" fillId="8" borderId="14" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <xf numFmtId="0" fontId="0" fillId="9" borderId="13" xfId="0" applyFill="1" applyBorder="1"/>
-    <xf numFmtId="168" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="168" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFill="1"/>
     <xf numFmtId="167" fontId="0" fillId="9" borderId="14" xfId="2" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <xf numFmtId="0" fontId="26" fillId="0" borderId="8" xfId="0" applyFont="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="1" xfId="3" quotePrefix="1" applyFont="1" applyAlignment="1"/>
+    <xf numFmtId="0" fontId="41" fillId="0" borderId="1" xfId="3" applyFont="1" applyAlignment="1"/>
     <xf numFmtId="0" fontId="14" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="168" fontId="44" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1"/>
   </cellXfs>
   <cellStyles count="12">
     <cellStyle name="Currency" xfId="1" builtinId="4"/>
@@ -1969,13 +1970,39 @@
   <dxfs count="104">
     <dxf>
       <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <color theme="0" tint="-0.499984740745262"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF00B050"/>
       </font>
     </dxf>
     <dxf>
       <font>
         <b/>
         <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0" tint="-0.499984740745262"/>
       </font>
     </dxf>
     <dxf>
@@ -1992,6 +2019,58 @@
           <bgColor theme="5" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0" tint="-0.499984740745262"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF00B050"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0" tint="-0.499984740745262"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FFFF0000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF00B050"/>
+      </font>
     </dxf>
     <dxf>
       <font>
@@ -2032,7 +2111,28 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FFFF0000"/>
+      </font>
+      <fill>
+        <patternFill>
+          <bgColor theme="5" tint="0.79998168889431442"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
         <color rgb="FF00B050"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <color theme="0" tint="-0.499984740745262"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
+        <b/>
+        <i val="0"/>
       </font>
     </dxf>
     <dxf>
@@ -2044,6 +2144,11 @@
           <bgColor theme="5" tint="0.79998168889431442"/>
         </patternFill>
       </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF00B050"/>
+      </font>
     </dxf>
     <dxf>
       <font>
@@ -2073,18 +2178,13 @@
     </dxf>
     <dxf>
       <font>
-        <color theme="0" tint="-0.499984740745262"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
         <b/>
         <i val="0"/>
       </font>
     </dxf>
     <dxf>
       <font>
-        <color rgb="FF00B050"/>
+        <color theme="0" tint="-0.499984740745262"/>
       </font>
     </dxf>
     <dxf>
@@ -2099,6 +2199,11 @@
     </dxf>
     <dxf>
       <font>
+        <color rgb="FF00B050"/>
+      </font>
+    </dxf>
+    <dxf>
+      <font>
         <color theme="0" tint="-0.499984740745262"/>
       </font>
     </dxf>
@@ -2106,11 +2211,6 @@
       <font>
         <b/>
         <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF00B050"/>
       </font>
     </dxf>
     <dxf>
@@ -2125,107 +2225,8 @@
     </dxf>
     <dxf>
       <font>
-        <color theme="0" tint="-0.499984740745262"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
         <color rgb="FF00B050"/>
       </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0" tint="-0.499984740745262"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF00B050"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0" tint="-0.499984740745262"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF00B050"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
-    </dxf>
-    <dxf>
-      <font>
-        <color theme="0" tint="-0.499984740745262"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <b/>
-        <i val="0"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FF00B050"/>
-      </font>
-    </dxf>
-    <dxf>
-      <font>
-        <color rgb="FFFF0000"/>
-      </font>
-      <fill>
-        <patternFill>
-          <bgColor theme="5" tint="0.79998168889431442"/>
-        </patternFill>
-      </fill>
     </dxf>
     <dxf>
       <font>
@@ -5928,10 +5929,10 @@
       <c r="K7" s="15"/>
     </row>
     <row r="8" spans="2:11" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B8" s="87" t="s">
+      <c r="B8" s="111" t="s">
         <v>20</v>
       </c>
-      <c r="C8" s="87"/>
+      <c r="C8" s="111"/>
     </row>
     <row r="9" spans="2:11" x14ac:dyDescent="0.3">
       <c r="B9" s="62"/>
@@ -6261,10 +6262,10 @@
       <c r="K30" s="37"/>
     </row>
     <row r="31" spans="2:12" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B31" s="87" t="s">
+      <c r="B31" s="111" t="s">
         <v>61</v>
       </c>
-      <c r="C31" s="87"/>
+      <c r="C31" s="111"/>
     </row>
     <row r="32" spans="2:12" x14ac:dyDescent="0.3">
       <c r="B32" s="36"/>
@@ -6479,10 +6480,10 @@
       <c r="K42" s="37"/>
     </row>
     <row r="43" spans="2:11" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B43" s="87" t="s">
+      <c r="B43" s="111" t="s">
         <v>67</v>
       </c>
-      <c r="C43" s="87"/>
+      <c r="C43" s="111"/>
     </row>
     <row r="45" spans="2:11" ht="15" thickBot="1" x14ac:dyDescent="0.35">
       <c r="B45" s="35" t="s">
@@ -6499,25 +6500,25 @@
       <c r="G46" s="45"/>
     </row>
     <row r="47" spans="2:11" ht="15" thickTop="1" x14ac:dyDescent="0.3">
-      <c r="B47" s="90" t="s">
+      <c r="B47" s="87" t="s">
         <v>173</v>
       </c>
-      <c r="C47" s="94"/>
-      <c r="F47" s="96"/>
-      <c r="G47" s="97" t="s">
+      <c r="C47" s="91"/>
+      <c r="F47" s="93"/>
+      <c r="G47" s="94" t="s">
         <v>70</v>
       </c>
-      <c r="H47" s="98" t="s">
+      <c r="H47" s="95" t="s">
         <v>172</v>
       </c>
       <c r="K47" s="2"/>
     </row>
     <row r="48" spans="2:11" x14ac:dyDescent="0.3">
-      <c r="B48" s="91" t="str">
+      <c r="B48" s="88" t="str">
         <f>$J$59</f>
         <v>Effective Federal Income Tax</v>
       </c>
-      <c r="C48" s="94">
+      <c r="C48" s="91">
         <f xml:space="preserve"> $K$64</f>
         <v>10589</v>
       </c>
@@ -6531,26 +6532,26 @@
 )</f>
         <v>= $K$64</v>
       </c>
-      <c r="F48" s="108" t="str">
+      <c r="F48" s="105" t="str">
         <f xml:space="preserve"> $B$39</f>
         <v>Total Gross Income:</v>
       </c>
-      <c r="G48" s="109">
+      <c r="G48" s="106">
         <f xml:space="preserve"> $C$39</f>
         <v>99000</v>
       </c>
-      <c r="H48" s="110">
+      <c r="H48" s="107">
         <f t="shared" ref="H48" si="2">$G48/$G$48</f>
         <v>1</v>
       </c>
       <c r="K48" s="2"/>
     </row>
     <row r="49" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B49" s="91" t="str">
+      <c r="B49" s="88" t="str">
         <f>$B$91</f>
         <v>Long Term Capital Gain Tax (LTCG)</v>
       </c>
-      <c r="C49" s="94">
+      <c r="C49" s="91">
         <f xml:space="preserve"> $C$111</f>
         <v>1050</v>
       </c>
@@ -6564,26 +6565,26 @@
 )</f>
         <v>= $C$111</v>
       </c>
-      <c r="F49" s="111"/>
-      <c r="G49" s="112"/>
-      <c r="H49" s="113"/>
+      <c r="F49" s="108"/>
+      <c r="G49" s="109"/>
+      <c r="H49" s="110"/>
       <c r="K49" s="2"/>
     </row>
     <row r="50" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B50" s="90" t="s">
+      <c r="B50" s="87" t="s">
         <v>170</v>
       </c>
-      <c r="C50" s="94"/>
+      <c r="C50" s="91"/>
       <c r="D50" s="61"/>
-      <c r="F50" s="99" t="str">
+      <c r="F50" s="96" t="str">
         <f>B55</f>
         <v>Total Tax Estimate:</v>
       </c>
-      <c r="G50" s="100">
+      <c r="G50" s="97">
         <f>C55</f>
         <v>17759</v>
       </c>
-      <c r="H50" s="101">
+      <c r="H50" s="98">
         <f>$G50/$G$48</f>
         <v>0.1793838383838384</v>
       </c>
@@ -6601,11 +6602,11 @@
       <c r="K50" s="2"/>
     </row>
     <row r="51" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B51" s="91" t="str">
+      <c r="B51" s="88" t="str">
         <f>$J$119</f>
         <v>Medicare Net Investment Income Tax (NIIT)</v>
       </c>
-      <c r="C51" s="94">
+      <c r="C51" s="91">
         <f xml:space="preserve"> $K$130</f>
         <v>0</v>
       </c>
@@ -6619,46 +6620,46 @@
 )</f>
         <v>= $K$130</v>
       </c>
-      <c r="F51" s="102" t="str">
+      <c r="F51" s="99" t="str">
         <f>$B$47</f>
         <v>Federal Income Taxes:</v>
       </c>
-      <c r="G51" s="103">
+      <c r="G51" s="100">
         <f>SUM($C$48:$C$49)</f>
         <v>11639</v>
       </c>
-      <c r="H51" s="104">
+      <c r="H51" s="101">
         <f t="shared" ref="H51:H55" si="3">$G51/$G$48</f>
         <v>0.11756565656565657</v>
       </c>
       <c r="K51" s="2"/>
     </row>
     <row r="52" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B52" s="90" t="s">
+      <c r="B52" s="87" t="s">
         <v>171</v>
       </c>
-      <c r="C52" s="94"/>
+      <c r="C52" s="91"/>
       <c r="D52" s="61"/>
-      <c r="F52" s="102" t="str">
+      <c r="F52" s="99" t="str">
         <f>$B$50</f>
         <v>Surtaxes:</v>
       </c>
-      <c r="G52" s="103">
+      <c r="G52" s="100">
         <f>SUM($C$51)</f>
         <v>0</v>
       </c>
-      <c r="H52" s="104">
+      <c r="H52" s="101">
         <f t="shared" si="3"/>
         <v>0</v>
       </c>
       <c r="K52" s="2"/>
     </row>
     <row r="53" spans="2:12" x14ac:dyDescent="0.3">
-      <c r="B53" s="91" t="str">
+      <c r="B53" s="88" t="str">
         <f>$B$119</f>
         <v>Social Security Tax</v>
       </c>
-      <c r="C53" s="94">
+      <c r="C53" s="91">
         <f xml:space="preserve"> $C$126</f>
         <v>4960</v>
       </c>
@@ -6672,26 +6673,26 @@
 )</f>
         <v>= $C$126</v>
       </c>
-      <c r="F53" s="102" t="str">
+      <c r="F53" s="99" t="str">
         <f>$B$52</f>
         <v>Payrol Taxes:</v>
       </c>
-      <c r="G53" s="103">
+      <c r="G53" s="100">
         <f>SUM($C$53:$C$54)</f>
         <v>6120</v>
       </c>
-      <c r="H53" s="104">
+      <c r="H53" s="101">
         <f t="shared" si="3"/>
         <v>6.1818181818181821E-2</v>
       </c>
       <c r="K53" s="2"/>
     </row>
     <row r="54" spans="2:12" ht="15.6" x14ac:dyDescent="0.3">
-      <c r="B54" s="92" t="str">
+      <c r="B54" s="89" t="str">
         <f>$F$119</f>
         <v>Medicare Wages Tax</v>
       </c>
-      <c r="C54" s="95">
+      <c r="C54" s="92">
         <f xml:space="preserve"> $G$129</f>
         <v>1160</v>
       </c>
@@ -6705,28 +6706,28 @@
 )</f>
         <v>= $G$129</v>
       </c>
-      <c r="F54" s="111"/>
-      <c r="G54" s="112"/>
-      <c r="H54" s="113"/>
+      <c r="F54" s="108"/>
+      <c r="G54" s="109"/>
+      <c r="H54" s="110"/>
       <c r="J54" s="33"/>
       <c r="K54" s="34"/>
     </row>
     <row r="55" spans="2:12" ht="16.2" thickBot="1" x14ac:dyDescent="0.35">
-      <c r="B55" s="93" t="s">
+      <c r="B55" s="90" t="s">
         <v>72</v>
       </c>
-      <c r="C55" s="94">
+      <c r="C55" s="115">
         <f>SUM(C48:C54)</f>
         <v>17759</v>
       </c>
-      <c r="F55" s="105" t="s">
+      <c r="F55" s="102" t="s">
         <v>71</v>
       </c>
-      <c r="G55" s="106">
+      <c r="G55" s="103">
         <f xml:space="preserve"> $G$48 - $G$50</f>
         <v>81241</v>
       </c>
-      <c r="H55" s="107">
+      <c r="H55" s="104">
         <f t="shared" si="3"/>
         <v>0.82061616161616158</v>
       </c>
@@ -7799,12 +7800,12 @@
       <c r="B116" s="15" t="s">
         <v>165</v>
       </c>
-      <c r="C116" s="88" t="s">
+      <c r="C116" s="112" t="s">
         <v>166</v>
       </c>
-      <c r="D116" s="89"/>
-      <c r="E116" s="89"/>
-      <c r="F116" s="89"/>
+      <c r="D116" s="113"/>
+      <c r="E116" s="113"/>
+      <c r="F116" s="113"/>
       <c r="G116" s="15"/>
       <c r="H116" s="15"/>
       <c r="J116" s="15" t="s">
@@ -8209,19 +8210,19 @@
       <formula>(H40 &lt;&gt; InRangeLabelCell)</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="I50">
+    <cfRule type="expression" dxfId="42" priority="1">
+      <formula>(I50 &lt;&gt; InRangeLabelCell)</formula>
+    </cfRule>
+  </conditionalFormatting>
   <conditionalFormatting sqref="L27">
-    <cfRule type="expression" dxfId="42" priority="6">
+    <cfRule type="expression" dxfId="41" priority="6">
       <formula>(L27 &lt;&gt; InRangeLabelCell)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L121">
-    <cfRule type="expression" dxfId="41" priority="3">
+    <cfRule type="expression" dxfId="40" priority="3">
       <formula>(L121 &lt;&gt; InRangeLabelCell)</formula>
-    </cfRule>
-  </conditionalFormatting>
-  <conditionalFormatting sqref="I50">
-    <cfRule type="expression" dxfId="40" priority="1">
-      <formula>(I50 &lt;&gt; InRangeLabelCell)</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="3">
@@ -16109,11 +16110,11 @@
   </sheetData>
   <phoneticPr fontId="40" type="noConversion"/>
   <conditionalFormatting sqref="C8">
-    <cfRule type="expression" dxfId="39" priority="49">
+    <cfRule type="expression" dxfId="39" priority="50">
+      <formula xml:space="preserve"> ($C$8 = SelectionValidLabelCell)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="38" priority="49">
       <formula xml:space="preserve"> ($C$8 &lt;&gt; SelectionValidLabelCell)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="38" priority="50">
-      <formula xml:space="preserve"> ($C$8 = SelectionValidLabelCell)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C10:C13">
@@ -16125,18 +16126,18 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C18">
-    <cfRule type="expression" dxfId="35" priority="41">
+    <cfRule type="expression" dxfId="35" priority="42">
+      <formula xml:space="preserve"> ($C$18 = SelectionValidLabelCell)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="34" priority="41">
       <formula xml:space="preserve"> ($C$18 &lt;&gt; SelectionValidLabelCell)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="34" priority="42">
-      <formula xml:space="preserve"> ($C$18 = SelectionValidLabelCell)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="C20:C22">
-    <cfRule type="cellIs" dxfId="33" priority="45" operator="equal">
+    <cfRule type="cellIs" dxfId="33" priority="46" operator="notEqual">
       <formula>TRUE</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="32" priority="46" operator="notEqual">
+    <cfRule type="cellIs" dxfId="32" priority="45" operator="equal">
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
@@ -16157,11 +16158,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J48">
-    <cfRule type="expression" dxfId="27" priority="38">
+    <cfRule type="expression" dxfId="27" priority="40">
+      <formula xml:space="preserve"> ($J$48 = SelectionValidLabelCell)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="26" priority="38">
       <formula xml:space="preserve"> ($J$48 &lt;&gt; SelectionValidLabelCell)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="26" priority="40">
-      <formula xml:space="preserve"> ($J$48 = SelectionValidLabelCell)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="J50:J63">
@@ -16173,11 +16174,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K68">
-    <cfRule type="expression" dxfId="23" priority="37">
+    <cfRule type="expression" dxfId="23" priority="39">
+      <formula xml:space="preserve"> ($K$68 = SelectionValidLabelCell)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="22" priority="37">
       <formula xml:space="preserve"> ($K$68 &lt;&gt; SelectionValidLabelCell)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="22" priority="39">
-      <formula xml:space="preserve"> ($K$68 = SelectionValidLabelCell)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="K70:K83">
@@ -16205,11 +16206,11 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L16">
-    <cfRule type="expression" dxfId="15" priority="57">
+    <cfRule type="expression" dxfId="15" priority="59">
+      <formula xml:space="preserve"> ($L$16 = SelectionValidLabelCell)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="14" priority="57">
       <formula xml:space="preserve"> ($L$16 &lt;&gt; SelectionValidLabelCell)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="14" priority="59">
-      <formula xml:space="preserve"> ($L$16 = SelectionValidLabelCell)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L18:L44">
@@ -16221,18 +16222,18 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L108">
-    <cfRule type="expression" dxfId="11" priority="29">
+    <cfRule type="expression" dxfId="11" priority="30">
+      <formula xml:space="preserve"> ($L$108 = SelectionValidLabelCell)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="10" priority="29">
       <formula xml:space="preserve"> ($L$108 &lt;&gt; SelectionValidLabelCell)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="10" priority="30">
-      <formula xml:space="preserve"> ($L$108 = SelectionValidLabelCell)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L110:L195">
-    <cfRule type="cellIs" dxfId="9" priority="27" operator="equal">
+    <cfRule type="cellIs" dxfId="9" priority="28" operator="notEqual">
       <formula>TRUE</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="8" priority="28" operator="notEqual">
+    <cfRule type="cellIs" dxfId="8" priority="27" operator="equal">
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
@@ -16245,27 +16246,27 @@
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L222:L247">
-    <cfRule type="cellIs" dxfId="5" priority="19" operator="equal">
+    <cfRule type="cellIs" dxfId="5" priority="20" operator="notEqual">
       <formula>TRUE</formula>
     </cfRule>
-    <cfRule type="cellIs" dxfId="4" priority="20" operator="notEqual">
+    <cfRule type="cellIs" dxfId="4" priority="19" operator="equal">
       <formula>TRUE</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L252:M252">
-    <cfRule type="expression" dxfId="3" priority="3">
+    <cfRule type="expression" dxfId="3" priority="4">
+      <formula xml:space="preserve"> (L$252 = SelectionValidLabelCell)</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="2" priority="3">
       <formula xml:space="preserve"> (L$252 &lt;&gt; SelectionValidLabelCell)</formula>
-    </cfRule>
-    <cfRule type="expression" dxfId="2" priority="4">
-      <formula xml:space="preserve"> (L$252 = SelectionValidLabelCell)</formula>
     </cfRule>
   </conditionalFormatting>
   <conditionalFormatting sqref="L254:M291">
-    <cfRule type="cellIs" dxfId="1" priority="1" operator="equal">
+    <cfRule type="cellIs" dxfId="1" priority="2" operator="equal">
+      <formula>FALSE</formula>
+    </cfRule>
+    <cfRule type="cellIs" dxfId="0" priority="1" operator="equal">
       <formula>TRUE</formula>
-    </cfRule>
-    <cfRule type="cellIs" dxfId="0" priority="2" operator="equal">
-      <formula>FALSE</formula>
     </cfRule>
   </conditionalFormatting>
   <dataValidations disablePrompts="1" count="3">

</xml_diff>